<commit_message>
docs(stage20): audit IT project management evidence
</commit_message>
<xml_diff>
--- a/reports/stage20/it-project-management/WORKSPHERE_PROJECT_MANAGEMENT_CALCULATIONS.xlsx
+++ b/reports/stage20/it-project-management/WORKSPHERE_PROJECT_MANAGEMENT_CALCULATIONS.xlsx
@@ -18,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +39,13 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +64,12 @@
         <bgColor rgb="00FFF2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E9ECEF"/>
+        <bgColor rgb="00E9ECEF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,6 +100,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -603,11 +629,13 @@
       <c r="G2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>0.11</v>
+      <c r="H2" s="6">
+        <f>(E2+4*F2+G2)/6</f>
+        <v/>
+      </c>
+      <c r="I2" s="7">
+        <f>((G2-E2)/6)^2</f>
+        <v/>
       </c>
       <c r="J2" s="2" t="n">
         <v>3</v>
@@ -676,11 +704,13 @@
       <c r="G3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>0.11</v>
+      <c r="H3" s="6">
+        <f>(E3+4*F3+G3)/6</f>
+        <v/>
+      </c>
+      <c r="I3" s="7">
+        <f>((G3-E3)/6)^2</f>
+        <v/>
       </c>
       <c r="J3" s="2" t="n">
         <v>4</v>
@@ -749,11 +779,13 @@
       <c r="G4" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>0.11</v>
+      <c r="H4" s="6">
+        <f>(E4+4*F4+G4)/6</f>
+        <v/>
+      </c>
+      <c r="I4" s="7">
+        <f>((G4-E4)/6)^2</f>
+        <v/>
       </c>
       <c r="J4" s="2" t="n">
         <v>4</v>
@@ -822,11 +854,13 @@
       <c r="G5" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>0.11</v>
+      <c r="H5" s="6">
+        <f>(E5+4*F5+G5)/6</f>
+        <v/>
+      </c>
+      <c r="I5" s="7">
+        <f>((G5-E5)/6)^2</f>
+        <v/>
       </c>
       <c r="J5" s="2" t="n">
         <v>5</v>
@@ -895,11 +929,13 @@
       <c r="G6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>0.11</v>
+      <c r="H6" s="8">
+        <f>(E6+4*F6+G6)/6</f>
+        <v/>
+      </c>
+      <c r="I6" s="9">
+        <f>((G6-E6)/6)^2</f>
+        <v/>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
@@ -968,11 +1004,13 @@
       <c r="G7" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="H7" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0.44</v>
+      <c r="H7" s="8">
+        <f>(E7+4*F7+G7)/6</f>
+        <v/>
+      </c>
+      <c r="I7" s="9">
+        <f>((G7-E7)/6)^2</f>
+        <v/>
       </c>
       <c r="J7" s="4" t="n">
         <v>12</v>
@@ -1041,11 +1079,13 @@
       <c r="G8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0.11</v>
+      <c r="H8" s="6">
+        <f>(E8+4*F8+G8)/6</f>
+        <v/>
+      </c>
+      <c r="I8" s="7">
+        <f>((G8-E8)/6)^2</f>
+        <v/>
       </c>
       <c r="J8" s="2" t="n">
         <v>5</v>
@@ -1114,11 +1154,13 @@
       <c r="G9" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H9" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>0.44</v>
+      <c r="H9" s="6">
+        <f>(E9+4*F9+G9)/6</f>
+        <v/>
+      </c>
+      <c r="I9" s="7">
+        <f>((G9-E9)/6)^2</f>
+        <v/>
       </c>
       <c r="J9" s="2" t="n">
         <v>14</v>
@@ -1187,11 +1229,13 @@
       <c r="G10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>0.11</v>
+      <c r="H10" s="8">
+        <f>(E10+4*F10+G10)/6</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>((G10-E10)/6)^2</f>
+        <v/>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
@@ -1260,11 +1304,13 @@
       <c r="G11" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H11" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>0.11</v>
+      <c r="H11" s="6">
+        <f>(E11+4*F11+G11)/6</f>
+        <v/>
+      </c>
+      <c r="I11" s="7">
+        <f>((G11-E11)/6)^2</f>
+        <v/>
       </c>
       <c r="J11" s="2" t="n">
         <v>6</v>
@@ -1333,11 +1379,13 @@
       <c r="G12" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>0.11</v>
+      <c r="H12" s="8">
+        <f>(E12+4*F12+G12)/6</f>
+        <v/>
+      </c>
+      <c r="I12" s="9">
+        <f>((G12-E12)/6)^2</f>
+        <v/>
       </c>
       <c r="J12" s="4" t="n">
         <v>4</v>
@@ -1406,11 +1454,13 @@
       <c r="G13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>0.11</v>
+      <c r="H13" s="6">
+        <f>(E13+4*F13+G13)/6</f>
+        <v/>
+      </c>
+      <c r="I13" s="7">
+        <f>((G13-E13)/6)^2</f>
+        <v/>
       </c>
       <c r="J13" s="2" t="n">
         <v>4</v>
@@ -1479,11 +1529,13 @@
       <c r="G14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>0.11</v>
+      <c r="H14" s="6">
+        <f>(E14+4*F14+G14)/6</f>
+        <v/>
+      </c>
+      <c r="I14" s="7">
+        <f>((G14-E14)/6)^2</f>
+        <v/>
       </c>
       <c r="J14" s="2" t="n">
         <v>3</v>
@@ -1552,11 +1604,13 @@
       <c r="G15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>0.11</v>
+      <c r="H15" s="6">
+        <f>(E15+4*F15+G15)/6</f>
+        <v/>
+      </c>
+      <c r="I15" s="7">
+        <f>((G15-E15)/6)^2</f>
+        <v/>
       </c>
       <c r="J15" s="2" t="n">
         <v>3</v>
@@ -2038,7 +2092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2146,8 +2200,9 @@
       <c r="J2" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="K2" s="4" t="n">
-        <v>117</v>
+      <c r="K2" s="4">
+        <f>SUM(D2:J2)</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -2185,8 +2240,9 @@
       <c r="J3" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="K3" s="4" t="n">
-        <v>120</v>
+      <c r="K3" s="4">
+        <f>SUM(D3:J3)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -2224,8 +2280,9 @@
       <c r="J4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>120</v>
+      <c r="K4" s="4">
+        <f>SUM(D4:J4)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -2263,8 +2320,57 @@
       <c r="J5" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="K5" s="4" t="n">
-        <v>120</v>
+      <c r="K5" s="4">
+        <f>SUM(D5:J5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Tổng Giờ Công Cả Nhóm</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Tất cả vai trò</t>
+        </is>
+      </c>
+      <c r="C6" s="10">
+        <f>SUM(C2:C5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="10">
+        <f>SUM(D2:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="10">
+        <f>SUM(E2:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="10">
+        <f>SUM(F2:F5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="10">
+        <f>SUM(G2:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="10">
+        <f>SUM(H2:H5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="10">
+        <f>SUM(I2:I5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="10">
+        <f>SUM(J2:J5)</f>
+        <v/>
+      </c>
+      <c r="K6" s="10">
+        <f>SUM(K2:K5)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>